<commit_message>
Commiting work in progress
</commit_message>
<xml_diff>
--- a/tests/ragas_test_dataset.xlsx
+++ b/tests/ragas_test_dataset.xlsx
@@ -30,9 +30,6 @@
     <t>What are Google's main environmental goals for 2023?</t>
   </si>
   <si>
-    <t>Google's environmental goals for 2023 include carbon neutrality, increased renewable energy use, and reducing water consumption.</t>
-  </si>
-  <si>
     <t>Simple</t>
   </si>
   <si>
@@ -244,6 +241,14 @@
   </si>
   <si>
     <t>Reference Text</t>
+  </si>
+  <si>
+    <t>Google's main environmental goals for 2023 include:
+1. Helping individuals, cities, and partners collectively reduce 1 gigaton of carbon equivalent emissions annually by 2030.
+2. Continuing to enhance and launch sustainability product features, such as eco-friendly routing in Google Maps, which has already helped prevent significant carbon emissions.
+3. Expanding the availability of Google Earth Engine to provide reliable insights on environmental changes to businesses and governments worldwide.  
+4. Operating sustainably through initiatives like the all-electric, net water-positive Bay View campus, which incorporates circular design principles.
+These goals reflect Google's commitment to advancing sustainability through technology and collaboration.</t>
   </si>
 </sst>
 </file>
@@ -599,8 +604,8 @@
   <dimension ref="A1:D24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.5703125" customWidth="1"/>
-    <col min="2" max="2" width="35" customWidth="1"/>
+    <col min="1" max="1" width="45.7109375" customWidth="1"/>
+    <col min="2" max="2" width="54.7109375" customWidth="1"/>
     <col min="3" max="3" width="40.7109375" customWidth="1"/>
     <col min="4" max="4" width="11.42578125" customWidth="1"/>
   </cols>
@@ -613,332 +618,332 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="270" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>4</v>
+        <v>75</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="105" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>27</v>
-      </c>
       <c r="D3" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="75" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>9</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="90" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="C5" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="90" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>14</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="90" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="B8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="105" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" s="2" t="s">
+      <c r="D8" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="B9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="90" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" s="2" t="s">
+      <c r="D9" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="B10" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B10" s="2" t="s">
+      <c r="D10" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="B11" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="105" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+      <c r="B12" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="C12" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+      <c r="B13" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="C13" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="D13" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="105" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
+      <c r="B14" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="C14" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="120" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
+      <c r="B15" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="C15" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="90" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
+      <c r="B16" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="C16" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="D16" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="105" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
+      <c r="B17" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="C17" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="D17" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="90" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
+      <c r="B18" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="C18" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="D18" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="90" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
+      <c r="B19" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="C19" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="D19" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="90" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
+      <c r="B20" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="C20" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="D20" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D20" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A21" s="2" t="s">
+      <c r="B21" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="C21" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="D21" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D21" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
+      <c r="B22" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="C22" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="D22" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="D22" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="90" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
+      <c r="B23" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="C23" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="D23" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="D23" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="105" x14ac:dyDescent="0.25">
-      <c r="A24" s="2" t="s">
+      <c r="B24" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="C24" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C24" s="2" t="s">
-        <v>74</v>
-      </c>
       <c r="D24" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>